<commit_message>
Optimize analyst workspace and harden reviewed evidence boundaries
</commit_message>
<xml_diff>
--- a/DATA_QUALITY.xlsx
+++ b/DATA_QUALITY.xlsx
@@ -82248,7 +82248,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-17T17:58:26.052168+00:00</t>
+          <t>2026-10-18T20:02:23.655186+00:00</t>
         </is>
       </c>
     </row>
@@ -82448,7 +82448,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>2b9bd4ef427437f7c79678cc</t>
+          <t>33cc3a616435735e314b5eb1</t>
         </is>
       </c>
     </row>
@@ -82544,7 +82544,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>2026-10-17T17:58:26.812400+00:00</t>
+          <t>2026-10-18T20:02:24.333960+00:00</t>
         </is>
       </c>
     </row>
@@ -82568,7 +82568,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>2026-10-17T17:58:26.052168+00:00</t>
+          <t>2026-10-18T20:02:23.655186+00:00</t>
         </is>
       </c>
     </row>
@@ -82664,7 +82664,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>2026-10-17T17:58:27.092726+00:00</t>
+          <t>2026-10-18T20:02:24.641961+00:00</t>
         </is>
       </c>
     </row>
@@ -82760,7 +82760,7 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>2026-10-17T17:58:27.410376+00:00</t>
+          <t>2026-10-18T20:02:24.960971+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add native WebMCP workflows with durable Agent admission
</commit_message>
<xml_diff>
--- a/DATA_QUALITY.xlsx
+++ b/DATA_QUALITY.xlsx
@@ -82248,7 +82248,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T20:02:23.655186+00:00</t>
+          <t>2026-10-18T21:11:49.395606+00:00</t>
         </is>
       </c>
     </row>
@@ -82448,7 +82448,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>33cc3a616435735e314b5eb1</t>
+          <t>5fb4c047808c71233216b53a</t>
         </is>
       </c>
     </row>
@@ -82544,7 +82544,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T20:02:24.333960+00:00</t>
+          <t>2026-10-18T21:11:50.125862+00:00</t>
         </is>
       </c>
     </row>
@@ -82568,7 +82568,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T20:02:23.655186+00:00</t>
+          <t>2026-10-18T21:11:49.395606+00:00</t>
         </is>
       </c>
     </row>
@@ -82664,7 +82664,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T20:02:24.641961+00:00</t>
+          <t>2026-10-18T21:11:50.456861+00:00</t>
         </is>
       </c>
     </row>
@@ -82760,7 +82760,7 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T20:02:24.960971+00:00</t>
+          <t>2026-10-18T21:11:50.847856+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve bilingual analysis flow and harden recovery contracts
Preserve public-summary identity across streamed and durable regrouping,
batch translation at response boundaries, and align the English and Vietnamese
analysis interface while retaining the concurrent owner changes.

Separate lossless computational inputs from spreadsheet-safe exports, correct
ratio and population labels, retain rejected translator admissions for recovery,
and avoid unsupported usage estimates or duplicate cumulative token counts.

Keep pending prompt recovery independent across tabs, propagate refresh aborts,
preserve existing visitors' read/cancel access at capacity, and prevent cleanup
alarm starvation and WebSocket bypasses during deferred upgrades.

Regenerate canonical deliverables and cover the reviewed failure paths with
focused regressions, including ordered README generation markers.
</commit_message>
<xml_diff>
--- a/DATA_QUALITY.xlsx
+++ b/DATA_QUALITY.xlsx
@@ -82248,7 +82248,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T21:11:49.395606+00:00</t>
+          <t>2026-10-19T03:28:18.346528+00:00</t>
         </is>
       </c>
     </row>
@@ -82448,7 +82448,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>5fb4c047808c71233216b53a</t>
+          <t>2aad0c28d1757a95e5a58a45</t>
         </is>
       </c>
     </row>
@@ -82544,7 +82544,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T21:11:50.125862+00:00</t>
+          <t>2026-10-19T03:28:19.129203+00:00</t>
         </is>
       </c>
     </row>
@@ -82568,7 +82568,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T21:11:49.395606+00:00</t>
+          <t>2026-10-19T03:28:18.346528+00:00</t>
         </is>
       </c>
     </row>
@@ -82664,7 +82664,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T21:11:50.456861+00:00</t>
+          <t>2026-10-19T03:28:19.439199+00:00</t>
         </is>
       </c>
     </row>
@@ -82760,7 +82760,7 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>2026-10-18T21:11:50.847856+00:00</t>
+          <t>2026-10-19T03:28:19.820203+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove record tracing and simplify Agent summary flow
Remove record-source tracing from Dashboard, API and Agent/WebMCP tools.
Keep original English public summaries in both locales and reduce streaming
render and scroll work while preserving source events and history.

Resolve six findings from five full-source review lanes: runtime-owned client
cleanup, quoted-source UI authority, citation cleanup parity, unavailable brief
comparators, KPI sparkline names and observer session restoration. Preserve
source inputs, the template, calculations, accounting and historical eval pins.

Validate frontend checks/build, 30 Cloudflare tests and deployment dry run,
backend formatting/lint/types, generated contracts and submission readback,
plus targeted offline recovery, authority, lifecycle and draft checks.
</commit_message>
<xml_diff>
--- a/DATA_QUALITY.xlsx
+++ b/DATA_QUALITY.xlsx
@@ -82248,7 +82248,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T03:28:18.346528+00:00</t>
+          <t>2026-10-19T05:48:09.843244+00:00</t>
         </is>
       </c>
     </row>
@@ -82448,7 +82448,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>2aad0c28d1757a95e5a58a45</t>
+          <t>a484bfa6924c5c24209884e9</t>
         </is>
       </c>
     </row>
@@ -82544,7 +82544,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T03:28:19.129203+00:00</t>
+          <t>2026-10-19T05:48:10.674608+00:00</t>
         </is>
       </c>
     </row>
@@ -82568,7 +82568,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T03:28:18.346528+00:00</t>
+          <t>2026-10-19T05:48:09.843244+00:00</t>
         </is>
       </c>
     </row>
@@ -82664,7 +82664,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T03:28:19.439199+00:00</t>
+          <t>2026-10-19T05:48:10.975712+00:00</t>
         </is>
       </c>
     </row>
@@ -82760,7 +82760,7 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T03:28:19.820203+00:00</t>
+          <t>2026-10-19T05:48:11.315947+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>